<commit_message>
Conexion de la api portal pesca
</commit_message>
<xml_diff>
--- a/datasets.xlsx
+++ b/datasets.xlsx
@@ -5,17 +5,17 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jhuamanciza\Desktop\Apps\app_seguimiento_insumos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jhuamanciza\Desktop\Apps\app_gestion_insumos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12C9926D-B923-43F3-B46E-2F4CA1931876}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B34652CE-518A-4A5A-B1E6-EB3B6B4B148C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-4230" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="db_insumos" sheetId="1" r:id="rId1"/>
     <sheet name="db_ratios_planta_insumo" sheetId="2" r:id="rId2"/>
-    <sheet name="bd_cuota" sheetId="3" r:id="rId3"/>
+    <sheet name="db_cuota" sheetId="3" r:id="rId3"/>
     <sheet name="db_capacidad_instalada" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
@@ -459,7 +459,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2C03C665-0CE5-4950-B558-45C586062E94}" name="bd_insumos" displayName="bd_insumos" ref="A1:D73" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20" headerRowCellStyle="Normal 2" dataCellStyle="Normal 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2C03C665-0CE5-4950-B558-45C586062E94}" name="db_insumos" displayName="db_insumos" ref="A1:D73" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20" headerRowCellStyle="Normal 2" dataCellStyle="Normal 2">
   <autoFilter ref="A1:D73" xr:uid="{2C03C665-0CE5-4950-B558-45C586062E94}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{263E8336-1D51-4111-9C56-77840C1CE105}" name="id_insumo" dataDxfId="19" dataCellStyle="Normal 2"/>
@@ -484,7 +484,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{22937465-9A69-4D88-ABFA-D3A771C272C4}" name="bd_cuota" displayName="bd_cuota" ref="A1:C2" totalsRowShown="0" headerRowDxfId="10" headerRowCellStyle="Normal 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{22937465-9A69-4D88-ABFA-D3A771C272C4}" name="db_cuota" displayName="db_cuota" ref="A1:C2" totalsRowShown="0" headerRowDxfId="10" headerRowCellStyle="Normal 2">
   <autoFilter ref="A1:C2" xr:uid="{22937465-9A69-4D88-ABFA-D3A771C272C4}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00924FDF-43DC-42C1-96FA-66DF0703D727}" name="cuota" dataDxfId="9" dataCellStyle="Normal 2"/>
@@ -776,7 +776,10 @@
   <dimension ref="A1:D73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="48" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -6291,8 +6294,10 @@
   <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="11.28515625" customWidth="1"/>
     <col min="3" max="3" width="20" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>